<commit_message>
Add tie-out and override log enhancements to separated tax packages
</commit_message>
<xml_diff>
--- a/bill-docs-k7m2v9/AllPro_Tax_2023.xlsx
+++ b/bill-docs-k7m2v9/AllPro_Tax_2023.xlsx
@@ -14,6 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P&amp;L_2023" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MONTHLY_2023" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LABOR_2023" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OVERRIDE_LOG_2023" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TIEOUT_2023" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +28,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +50,10 @@
     <font>
       <b val="1"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="007A0000"/>
     </font>
   </fonts>
   <fills count="3">
@@ -75,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -86,6 +92,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -45485,4 +45492,266 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Manual Override Log - 2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Warning: Changing classification may impact tax reporting. Confirm with tax professional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Manual Override Count</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>COUNTIF(CATEGORIZED_2023!$H:$H,"YES")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Total Amount in Overridden Transactions</t>
+        </is>
+      </c>
+      <c r="B6" s="2">
+        <f>SUMIFS(CATEGORIZED_2023!$C:$C,CATEGORIZED_2023!$H:$H,"YES")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Original Group</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Final Group</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Manual Override</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>Override Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <f>IFERROR(FILTER(CATEGORIZED_2023!A:I,CATEGORIZED_2023!H:H="YES"),"No manual overrides")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="54" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Raw Credits Total</t>
+        </is>
+      </c>
+      <c r="B2" s="2">
+        <f>SUMIFS(RAW_2023!$C:$C,RAW_2023!$D:$D,"Credit")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Raw Debits Total</t>
+        </is>
+      </c>
+      <c r="B3" s="2">
+        <f>SUMIFS(RAW_2023!$C:$C,RAW_2023!$D:$D,"Debit")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Raw Net (Credits-Debits)</t>
+        </is>
+      </c>
+      <c r="B4" s="2">
+        <f>B2-B3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Categorized Revenue (Final Group)</t>
+        </is>
+      </c>
+      <c r="B5" s="2">
+        <f>SUMIFS(CATEGORIZED_2023!$C:$C,CATEGORIZED_2023!$G:$G,"Revenue")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Categorized COGS (Final Group)</t>
+        </is>
+      </c>
+      <c r="B6" s="2">
+        <f>SUMIFS(CATEGORIZED_2023!$C:$C,CATEGORIZED_2023!$G:$G,"COGS")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Categorized Expense (Final Group)</t>
+        </is>
+      </c>
+      <c r="B7" s="2">
+        <f>SUMIFS(CATEGORIZED_2023!$C:$C,CATEGORIZED_2023!$G:$G,"Expense")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Categorized Non-Deductible (Final Group)</t>
+        </is>
+      </c>
+      <c r="B8" s="2">
+        <f>SUMIFS(CATEGORIZED_2023!$C:$C,CATEGORIZED_2023!$G:$G,"Non-Deductible")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Categorized Total Counted</t>
+        </is>
+      </c>
+      <c r="B9" s="2">
+        <f>B5+B6+B7+B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Coverage Check (Raw total vs Categorized total)</t>
+        </is>
+      </c>
+      <c r="B10" s="2">
+        <f>ABS((B2+B3)-B9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Note: 2023 source is internal workbook (no bank statement balances available for beginning/ending tie-out).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>